<commit_message>
Plans update live on the site; old @smartmarket.dev emails move to @smartplaze.com
- /subscriptions and /sell read the plans without the 5-minute page cache
  (the API keeps its Redis copy and clears it on every plan change), so an
  admin edit shows at once
- scripts/rebrand-emails.js moves @smartmarket.dev accounts to
  @smartplaze.com and guest placeholders to @guest.smartplaze.invalid,
  refusing on any clash; seed, catalog import and create-user now use the
  SmartPlaze domain and default names; test workbook and docs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SmartPlaze_Test_Scenarios.xlsx
+++ b/docs/SmartPlaze_Test_Scenarios.xlsx
@@ -1304,6 +1304,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -1359,6 +1360,8 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="26.25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1751,6 +1754,7 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -3298,12 +3302,12 @@
       <c r="E28" s="3" t="inlineStr">
         <is>
           <t>1.
-Register with test@smartmarket.dev.</t>
+Register with test@smartplaze.com.</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>test@smartmarket.dev</t>
+          <t>test@smartplaze.com</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -3354,7 +3358,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>buyer@smartmarket.dev / BuyerPass123</t>
+          <t>buyer@smartplaze.com / BuyerPass123</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -3405,7 +3409,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>buyer@smartmarket.dev / wrong</t>
+          <t>buyer@smartplaze.com / wrong</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -7662,7 +7666,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>tech.elite@smartmarket.dev / Seller123! buying Smart Trust items</t>
+          <t>tech.elite@smartplaze.com / Seller123! buying Smart Trust items</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -8098,7 +8102,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>tech.elite@smartmarket.dev</t>
+          <t>tech.elite@smartplaze.com</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr">
@@ -8220,6 +8224,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -8250,7 +8255,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>test@smartmarket.dev</t>
+          <t>test@smartplaze.com</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -8272,7 +8277,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>accountant@smartmarket.dev</t>
+          <t>accountant@smartplaze.com</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -8294,7 +8299,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>cs@smartmarket.dev</t>
+          <t>cs@smartplaze.com</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -8316,7 +8321,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>buyer@smartmarket.dev</t>
+          <t>buyer@smartplaze.com</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -8338,7 +8343,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>smarttrust@smartmarket.dev</t>
+          <t>smarttrust@smartplaze.com</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -8360,7 +8365,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>tech.elite@smartmarket.dev</t>
+          <t>tech.elite@smartplaze.com</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -8374,6 +8379,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="16.85" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>

</xml_diff>